<commit_message>
Updated report for Interim Report #2
</commit_message>
<xml_diff>
--- a/projects/nas-sos-capstone/cameo_models/print/requirements-review.xlsx
+++ b/projects/nas-sos-capstone/cameo_models/print/requirements-review.xlsx
@@ -9,16 +9,18 @@
   <sheets>
     <sheet name="Decomposition" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Stakeholder reqs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="System reqs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sub-system HLRs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="About" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Objectives" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Stakeholder reqs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="System reqs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sub-system HLRs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="About" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Decomposition'!$A$1:$G$139</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stakeholder reqs'!$A$1:$K$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'System reqs'!$A$1:$P$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sub-system HLRs'!$A$1:$Q$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Objectives'!$A$1:$H$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stakeholder reqs'!$A$1:$K$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'System reqs'!$A$1:$P$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sub-system HLRs'!$A$1:$Q$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -186,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -248,6 +250,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4214,6 +4219,1645 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Objective row</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Trajectory impact</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Stakeholder requirements in the study</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Background / out of study</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>In-study system requirements reached</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>HLRs reached</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Review notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Fuel cost</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Crew cost</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Aircraft utilization</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Schedule integrity</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02, SN-AIR-03, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>SLR-CLR-04, SLR-CLR-13, SLR-INF-02, SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-05, HLR-OPS-06, HLR-ATC-05, HLR-ATC-08, HLR-ACF-04, HLR-ACF-05, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Passenger connections</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>SN-AIR-04 (out of study)</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>SLR-CLR-13, SLR-INF-02, SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-05, HLR-OPS-06, HLR-ATC-05, HLR-ATC-08, HLR-ACF-05, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Delay cost</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-03</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>SN-AIR-04 (out of study)</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-04, SLR-CLR-09, SLR-INF-07, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-04, HLR-CRW-05, HLR-OPS-01, HLR-OPS-06, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-04, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Dispatch reliability</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Flight Safety</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>SN-ATC-01</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>SN-PAX-01 (out of study)</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-06, SLR-CLR-01, SLR-CLR-02, SLR-INF-01, SLR-EXE-02</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-01, HLR-OPS-02, HLR-ATC-01, HLR-ATC-02, HLR-ATC-03, HLR-ATC-04, HLR-ACF-02, HLR-ACF-06</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Ticket price</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Travel time</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>SN-PAX-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Connection reliability</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>SN-PAX-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Schedule convenience</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Comfort</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>SN-PAX-03 (out of study)</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-07, HLR-ATC-07, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Disruption risk</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>SN-PAX-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>ATC / ANSP</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Safety/separation</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>SN-ATC-01</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-06, SLR-CLR-01, SLR-CLR-02, SLR-INF-01, SLR-EXE-02</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-01, HLR-OPS-02, HLR-ATC-01, HLR-ATC-02, HLR-ATC-03, HLR-ATC-04, HLR-ACF-02, HLR-ACF-06</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>ATC / ANSP</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>Sector workload</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>SN-ATC-04</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>SLR-CLR-15</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>HLR-ATC-06</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>ATC / ANSP</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>SN-ATC-02</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-06</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>HLR-OPS-02</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>ATC / ANSP</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Predictability</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>SN-ATC-03 (out of study)</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>ATC / ANSP</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>Delay (ATC-attributed)</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>SN-ATC-05 (out of study)</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>ATC / ANSP</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Traffic complexity</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>SN-ATC-04</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>SLR-CLR-15</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>HLR-ATC-06</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Gate utilization</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>SN-APT-01 (out of study)</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Runway utilization</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>SN-APT-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Surface congestion</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>SN-APT-03 (out of study)</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>Turnaround performance</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>SN-APT-01 (out of study)</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>Passenger throughput</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>SN-APT-01 (out of study)</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Flight Crew</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>SN-CRW-03, SN-CRW-06, SN-CRW-07</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>SN-CRW-01 (out of study), SN-CRW-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-07, SLR-CLR-01, SLR-CLR-02, SLR-CLR-10, SLR-INF-02, SLR-EXE-03, SLR-EXE-06</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-02, HLR-CRW-03, HLR-CRW-04, HLR-CRW-05, HLR-OPS-03, HLR-OPS-05, HLR-OPS-06, HLR-ATC-01, HLR-ATC-02, HLR-ATC-04, HLR-ATC-08, HLR-ACF-01, HLR-ACF-03, HLR-ACF-05, HLR-ACF-06, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Flight Crew</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Workload</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>SN-CRW-03, SN-CRW-08</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>SLR-CLR-04, SLR-CLR-10, SLR-INF-02, SLR-EXE-03, SLR-EXE-06</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-02, HLR-CRW-03, HLR-CRW-04, HLR-CRW-05, HLR-OPS-05, HLR-OPS-06, HLR-ATC-04, HLR-ATC-08, HLR-ACF-01, HLR-ACF-03, HLR-ACF-04, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Flight Crew</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Procedural compliance</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>SN-CRW-07, SN-CRW-08</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>SN-CRW-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-07, SLR-CLR-04</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-CRW-05, HLR-OPS-03, HLR-OPS-06, HLR-ACF-04, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Flight Crew</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Schedule/duty constraints</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-02</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>SN-CRW-05 (out of study)</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>SLR-INF-07, SLR-APT-04</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-04, HLR-OPS-06, HLR-APT-01, HLR-APT-02</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Flight Crew</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>Operational flexibility</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>SN-CRW-01 (out of study), SN-CRW-04 (out of study)</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Environmental / Societal</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>CO2</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>SN-ENV-01 (background)</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Environmental / Societal</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>NOx</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>SN-ENV-01 (background)</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Environmental / Societal</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>Contrail/climate effects</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>SN-ENV-01 (background)</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Environmental / Societal</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>Noise</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>SN-ENV-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Environmental / Societal</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>Local air quality</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>SN-AIR-01, SN-AIR-05</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>SN-ENV-01 (background)</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>SLR-PLN-01, SLR-PLN-02, SLR-CLR-09, SLR-CLR-13, SLR-INF-02, SLR-EXE-03, SLR-MEA-02</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>HLR-CRW-03, HLR-CRW-05, HLR-OPS-01, HLR-OPS-05, HLR-OPS-07, HLR-ATC-05, HLR-ATC-07, HLR-ATC-08, HLR-ACF-01, HLR-ACF-05</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Mission effectiveness</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr"/>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>(no requirement)</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr"/>
+      <c r="G39" s="13" t="inlineStr"/>
+      <c r="H39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Mission timing</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr"/>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>(no requirement)</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr"/>
+      <c r="G40" s="13" t="inlineStr"/>
+      <c r="H40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Fuel availability</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr"/>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>(no requirement)</t>
+        </is>
+      </c>
+      <c r="F41" s="13" t="inlineStr"/>
+      <c r="G41" s="13" t="inlineStr"/>
+      <c r="H41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>Airspace access</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr"/>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>SN-MIL-01 (out of study)</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr"/>
+      <c r="G42" s="22" t="inlineStr"/>
+      <c r="H42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>Operational security</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr"/>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>(no requirement)</t>
+        </is>
+      </c>
+      <c r="F43" s="13" t="inlineStr"/>
+      <c r="G43" s="13" t="inlineStr"/>
+      <c r="H43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>Military</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr"/>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>(no requirement)</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr"/>
+      <c r="G44" s="13" t="inlineStr"/>
+      <c r="H44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>(no objective row)</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>SN-AIR-06 (out of study)</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Regulator</t>
+        </is>
+      </c>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>(no objective row)</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>SN-GOV-01 (background)</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Regulator</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>(no objective row)</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>SN-GOV-02 (out of study)</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H47"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4305,7 +5949,7 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>Airline: Fuel cost; Airline: Delay cost</t>
+          <t>Airline: Fuel cost; Airline: Delay cost; Airline: Crew cost; Airline: Maintenance; Airline: Revenue; Passenger: Ticket price; Passenger: Schedule convenience; Passenger: Comfort; Flight Crew: Operational flexibility; Environmental / Societal: CO2; Environmental / Societal: NOx; Environmental / Societal: Contrail/climate effects; Environmental / Societal: Noise; Environmental / Societal: Local air quality</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr">
@@ -4335,7 +5979,7 @@
       </c>
       <c r="J2" s="13" t="inlineStr">
         <is>
-          <t>In the study: the planned cruise altitude and speed are what a conflict resolution takes the aircraft away from, so this is what the experiment scores a resolution against. The owner struck 'at its lowest operating cost' (hand review 2026-10-11): what the airline optimizes for is the airline's own business. The owner struck ', so that the flight is flown within safety and capacity limits' (hand review 2026-10-20).</t>
+          <t>In the study: the planned cruise altitude and speed are what a conflict resolution takes the aircraft away from, so this is what the experiment scores a resolution against. The owner struck 'at its lowest operating cost' (hand review 2026-10-11): what the airline optimizes for is the airline's own business. The owner struck ', so that the flight is flown within safety and capacity limits' (hand review 2026-10-20). Objective rows added by the owner in the workbook review of 2026-10-22 (D-032): Airline: Crew cost; Airline: Maintenance; Airline: Revenue; Passenger: Ticket price; Passenger: Schedule convenience; Passenger: Comfort; Flight Crew: Operational flexibility; Environmental / Societal: CO2; Environmental / Societal: NOx; Environmental / Societal: Contrail/climate effects; Environmental / Societal: Noise; Environmental / Societal: Local air quality. Owner on 'Passenger: Ticket price' (2026-10-22): the airline sets prices from its costs, as represented in the fuel, time and maintenance impacts of its flight schedules as planned.</t>
         </is>
       </c>
       <c r="K2" s="13" t="n"/>
@@ -4358,7 +6002,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Airline: Schedule integrity; Airline: Aircraft utilization; Airline: Passenger connections</t>
+          <t>Airline: Schedule integrity; Airline: Aircraft utilization; Airline: Passenger connections; Airline: Dispatch reliability; Passenger: Travel time; Passenger: Connection reliability; Passenger: Disruption risk; ATC / ANSP: Predictability; ATC / ANSP: Delay (ATC-attributed); Airport: Gate utilization; Airport: Runway utilization; Airport: Surface congestion; Airport: Turnaround performance; Airport: Passenger throughput; Flight Crew: Schedule/duty constraints</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -4384,7 +6028,7 @@
       <c r="I3" s="13" t="inlineStr"/>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>In the study: the time side of the fuel-against-time trade, and the reason one flight's connections can outweigh its fuel (case D of the experiment). Owner's wording, hand review 2026-10-10.</t>
+          <t>In the study: the time side of the fuel-against-time trade, and the reason one flight's connections can outweigh its fuel (case D of the experiment). Owner's wording, hand review 2026-10-10. Objective rows added by the owner in the workbook review of 2026-10-22 (D-032): Airline: Dispatch reliability; Passenger: Travel time; Passenger: Connection reliability; Passenger: Disruption risk; ATC / ANSP: Predictability; ATC / ANSP: Delay (ATC-attributed); Airport: Gate utilization; Airport: Runway utilization; Airport: Surface congestion; Airport: Turnaround performance; Airport: Passenger throughput; Flight Crew: Schedule/duty constraints.</t>
         </is>
       </c>
       <c r="K3" s="13" t="n"/>
@@ -4513,7 +6157,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Airline: Fuel cost; Airline: Schedule integrity; Airline: Passenger connections</t>
+          <t>Airline: Fuel cost; Airline: Schedule integrity; Airline: Passenger connections; Flight Crew: Operational flexibility; Environmental / Societal: CO2; Environmental / Societal: NOx; Environmental / Societal: Contrail/climate effects; Environmental / Societal: Noise; Environmental / Societal: Local air quality</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -4538,12 +6182,12 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>schultz2012adaptiveClimb; coppenbarger1999climbPrediction</t>
+          <t>schultz2012adaptiveClimb; coppenbarger1999climbPrediction; kulkarni2019ctopSlotSubstitution</t>
         </is>
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>In the study: this is the requirement the experiment is about (knowledge/models/experiment-definition.md section 2). It is not met today: the controller does not receive weight or cost index. Owner's wording, hand review 2026-10-10.</t>
+          <t>In the study: this is the requirement the experiment is about (knowledge/models/experiment-definition.md section 2). Met today in part, before departure (owner, 2026-10-22): in the FAA's Collaborative Trajectory Options Program the airline submits a Trajectory Options Set, each route option carrying a Relative Trajectory Cost in equivalent ground-delay minutes, and the FAA's algorithm adds that cost to the assigned delay and picks the cheapest option (kulkarni2019ctopSlotSubstitution, p. 4). It is not met in tactical conflict resolution in cruise, the decision the study examines: the controller does not receive weight or cost index. Owner's wording, hand review 2026-10-10. Objective rows added by the owner in the workbook review of 2026-10-22 (D-032): Flight Crew: Operational flexibility; Environmental / Societal: CO2; Environmental / Societal: NOx; Environmental / Societal: Contrail/climate effects; Environmental / Societal: Noise; Environmental / Societal: Local air quality.</t>
         </is>
       </c>
       <c r="K6" s="13" t="n"/>
@@ -4619,7 +6263,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>ATC / ANSP: Safety/separation</t>
+          <t>ATC / ANSP: Safety/separation; Airline: Flight Safety</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -4649,7 +6293,7 @@
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>In the study: the hard constraint every resolution option must meet. It is never traded against cost (knowledge/models/experiment-definition.md section 6).</t>
+          <t>In the study: the hard constraint every resolution option must meet. It is never traded against cost (knowledge/models/experiment-definition.md section 6). Objective rows added by the owner in the workbook review of 2026-10-22 (D-032): Airline: Flight Safety.</t>
         </is>
       </c>
       <c r="K8" s="13" t="n"/>
@@ -5398,7 +7042,7 @@
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Environmental / Societal: CO2</t>
+          <t>Environmental / Societal: CO2; Environmental / Societal: NOx; Environmental / Societal: Contrail/climate effects; Environmental / Societal: Local air quality</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -5428,7 +7072,7 @@
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>In the study: CO2 is fuel burned times 3.16 (D-015), so the experiment's fuel column is also this stakeholder's column. 'Economics' was added by the owner (hand review 2026-10-10) and left standing in the second review. Owner (hand review 2026-10-20): 'This is currently in my cost, but not in my stakeholders. They're treated as background/input.' Tagged background (D-031).</t>
+          <t>In the study: CO2 is fuel burned times 3.16 (D-015), so the experiment's fuel column is also this stakeholder's column. 'Economics' was added by the owner (hand review 2026-10-10) and left standing in the second review. Owner (hand review 2026-10-20): 'This is currently in my cost, but not in my stakeholders. They're treated as background/input.' Tagged background (D-031). Objective rows added by the owner in the workbook review of 2026-10-22 (D-032): Environmental / Societal: NOx; Environmental / Societal: Contrail/climate effects; Environmental / Societal: Local air quality.</t>
         </is>
       </c>
       <c r="K23" s="13" t="n"/>
@@ -5451,7 +7095,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Environmental / Societal: Noise; Environmental / Societal: Community impacts</t>
+          <t>Environmental / Societal: Noise</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -5500,7 +7144,7 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Airport: Gate utilization; Airport: Turnaround performance</t>
+          <t>Airport: Gate utilization; Airport: Turnaround performance; Airport: Passenger throughput</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -5526,7 +7170,7 @@
       <c r="I25" s="13" t="inlineStr"/>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>Restored as out of study (D-031): the owner's hand review of 2026-10-20 keeps every stakeholder requirement of the first draft and makes the cut at the sub-system (HLR) tier. Text as on the 2026-10-10 print. Struck 2026-10-10: 'All of these are not D-007'.</t>
+          <t>Restored as out of study (D-031): the owner's hand review of 2026-10-20 keeps every stakeholder requirement of the first draft and makes the cut at the sub-system (HLR) tier. Text as on the 2026-10-10 print. Struck 2026-10-10: 'All of these are not D-007'. Objective rows added by the owner in the workbook review of 2026-10-22 (D-032): Airport: Passenger throughput.</t>
         </is>
       </c>
       <c r="K25" s="13" t="n"/>
@@ -5831,7 +7475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8990,7 +10634,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11306,110 +12950,120 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>Requirements review workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
-        <is>
-          <t>Generated 2026-10-20 22:25 from commit 1785b6c by tools/export_requirements_xlsx.py.</t>
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Generated 2026-10-22 21:42 from commit d0c723d by tools/export_requirements_xlsx.py.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Source of truth: the .sysml files in projects/nas-sos-capstone/cameo_models/ (D-006). This workbook is a derived copy: mark it up, then apply the changes to the .sysml files and regenerate.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Counts: 30 stakeholder requirements, 42 system requirements, 29 sub-system HLRs. The Coverage sheet counts each by scope and lists any trace gap.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr"/>
+      <c r="A5" s="25" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
         <is>
+          <t>Objectives sheet: reads the other way, from each objective row of knowledge/models/stakeholder-objective-ontology.md to the stakeholder requirements that name it (attribute objectiveRefs), and on to the in-study system requirements and HLRs below them. Bold objective: carried into the study. Grey: carried only by a background or out-of-study requirement. '(no requirement)': no stakeholder requirement names it. Requirements that name no objective row are listed at the end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
           <t>How the Decomposition sheet reads</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Left to right: stakeholder requirement (SN) -&gt; the system requirements (SLR) that answer it -&gt; the HLRs that come from each SLR. Merged cells span the rows beneath them.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>The trace is many-to-many, so an SLR that answers two stakeholder requirements appears under both, marked '(also answers ...)'. An HLR with two parents is marked '(also comes from ...)'.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>[IMPROVED] and orange fill: architectureState = improved, something today's NAS does not do (D-018). [GOAL] and italics: obligation = goal, written with 'should' (D-020).</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>[OUT OF STUDY], grey fill and grey text: studyScope = outOfStudy (D-031). Every stakeholder requirement of the first draft is kept, with the system requirements that answer it; the study's cut is made at the HLR tier, so these stop at the system level with '(no HLR: not carried into the study)'. [BACKGROUND] and lilac fill: a boundary actor's requirement the study holds fixed and uses as input (the operating rules, the CO2 factor). '(no HLR: gap)' in red would be an in-study system requirement with nothing under it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
+          <t>[OUT OF STUDY], grey fill and grey text: studyScope = outOfStudy (D-031). Every stakeholder requirement of the first draft is kept, with the system requirements that answer it; the study's cut is made at the HLR tier, so these stop at the system level with '(no HLR: not carried into the study)'. [BACKGROUND] and lilac fill: a boundary actor's requirement the study holds fixed and uses as input (the operating rules, the CO2 factor). '(no HLR: gap)' in red would be an in-study system requirement with nothing under it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
           <t>Review status (from knowledge/models/requirements-and-traceability.md)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>In-study stakeholder and system requirements: hand-reviewed by the owner three times (D-020, D-021, D-031). Out-of-study ones: restored on 2026-10-20 from the 10-10 and 10-11 prints with the text they had when struck.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Sub-system HLRs: Claude's draft of 2026-10-11 (D-022), hand-reviewed by the owner on 2026-10-20 (D-031). Edits applied from a question on that print say so in their rationale and await the owner's confirmation; HLR-ACF-06 is new.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Every requirement has status = draft. Nothing is baselined.</t>
         </is>

</xml_diff>

<commit_message>
Experiment review w/#TODOs, Use Case & Sequence creation, requirement diagrams (which look really nice), a number of decisions, and follow-on updates.
</commit_message>
<xml_diff>
--- a/projects/nas-sos-capstone/cameo_models/print/requirements-review.xlsx
+++ b/projects/nas-sos-capstone/cameo_models/print/requirements-review.xlsx
@@ -16,7 +16,7 @@
     <sheet name="About" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Decomposition'!$A$1:$G$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Decomposition'!$A$1:$H$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Objectives'!$A$1:$H$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stakeholder reqs'!$A$1:$K$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'System reqs'!$A$1:$P$43</definedName>
@@ -188,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -243,7 +243,13 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -629,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -639,6 +645,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -672,7 +679,12 @@
           <t>Sub-system HLR (constituent system shall)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Objectives addressed</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Review notes</t>
         </is>
@@ -690,6 +702,7 @@
       <c r="E2" s="6" t="n"/>
       <c r="F2" s="6" t="n"/>
       <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -724,7 +737,12 @@
 (also comes from SLR-PLN-02, SLR-PLN-04)</t>
         </is>
       </c>
-      <c r="G3" s="13" t="n"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Fuel cost, Crew cost, Maintenance, Delay cost, Revenue, Ticket price, Schedule convenience, Comfort, Operational flexibility, CO2, NOx, Contrail/climate effects, Noise, Local air quality</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n"/>
@@ -750,7 +768,8 @@
 (also comes from SLR-PLN-01, SLR-PLN-04)</t>
         </is>
       </c>
-      <c r="G4" s="13" t="n"/>
+      <c r="G4" s="14" t="n"/>
+      <c r="H4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n"/>
@@ -777,7 +796,8 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n"/>
+      <c r="G5" s="14" t="n"/>
+      <c r="H5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n"/>
@@ -794,7 +814,8 @@
           <t>Air traffic control shall answer each flight crew request for a route, altitude or speed change with an approval, an amended clearance or 'unable'.</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n"/>
@@ -821,7 +842,8 @@
 (also comes from SLR-CLR-09)</t>
         </is>
       </c>
-      <c r="G7" s="13" t="n"/>
+      <c r="G7" s="14" t="n"/>
+      <c r="H7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n"/>
@@ -839,7 +861,8 @@
 (also comes from SLR-PLN-07)</t>
         </is>
       </c>
-      <c r="G8" s="13" t="n"/>
+      <c r="G8" s="14" t="n"/>
+      <c r="H8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n"/>
@@ -856,7 +879,8 @@
           <t>The flight management system shall predict the flight's arrival time, fuel at the destination, optimum altitude and maximum altitude from the entered weights, the cost index and the forecast winds.</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n"/>
+      <c r="G9" s="14" t="n"/>
+      <c r="H9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n"/>
@@ -874,7 +898,8 @@
 (also comes from SLR-INF-02)</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n"/>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -900,7 +925,8 @@
           <t>Flight operations shall report each flight's fuel burned and its CO2 emitted at 3.16 kg of CO2 per kg of fuel.</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -935,7 +961,12 @@
 (also comes from SLR-EXE-06, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Aircraft utilization, Schedule integrity, Passenger connections, Dispatch reliability, Travel time, Connection reliability, Disruption risk, Predictability, Delay (ATC-attributed), Gate utilization, Runway utilization, Surface congestion, Turnaround performance, Passenger throughput, Schedule/duty constraints</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n"/>
@@ -953,7 +984,8 @@
 (also comes from SLR-CLR-04, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G13" s="13" t="n"/>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n"/>
@@ -975,7 +1007,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G14" s="13" t="n"/>
+      <c r="G14" s="14" t="n"/>
+      <c r="H14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n"/>
@@ -1000,7 +1033,8 @@
           <t>Airport operations shall have each aircraft fuelled, loaded and sealed by its scheduled off-block time.</t>
         </is>
       </c>
-      <c r="G15" s="13" t="n"/>
+      <c r="G15" s="14" t="n"/>
+      <c r="H15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n"/>
@@ -1018,7 +1052,8 @@
 (also comes from SLR-PLN-07)</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -1040,7 +1075,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1070,7 +1106,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Schedule integrity, Delay cost</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n"/>
@@ -1097,7 +1138,8 @@
 (also comes from SLR-INF-07, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G19" s="13" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="14" t="n"/>
@@ -1115,7 +1157,8 @@
 (also comes from SLR-INF-07, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G20" s="13" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="13" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n"/>
@@ -1132,7 +1175,8 @@
           <t>The aircraft communication system shall carry voice and data between the flight crew and both air traffic control and the dispatcher for the whole flight.</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="14" t="n"/>
@@ -1159,7 +1203,8 @@
 (also comes from SLR-EXE-06, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -1177,7 +1222,8 @@
 (also comes from SLR-CLR-04, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1206,7 +1252,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n"/>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>Passenger connections, Delay cost</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1240,7 +1291,12 @@
           <t>[GOAL, IMPROVED] Air traffic control should choose, among the clearances that resolve a conflict and can be flown, the one with the lowest impact on the systems involved.</t>
         </is>
       </c>
-      <c r="G25" s="13" t="n"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Fuel cost, Schedule integrity, Passenger connections, Operational flexibility, CO2, NOx, Contrail/climate effects, Noise, Local air quality</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="n"/>
@@ -1266,7 +1322,8 @@
           <t>[IMPROVED] Flight operations shall make each flight's current gross weight, performance model, relative cost of flight time and connection priority available to the party that decides a change to that flight's trajectory.</t>
         </is>
       </c>
-      <c r="G26" s="13" t="n"/>
+      <c r="G26" s="14" t="n"/>
+      <c r="H26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="14" t="n"/>
@@ -1283,7 +1340,8 @@
           <t>[IMPROVED] ATC decision support shall use the best information available to it about each flight, including the gross weight, performance model, relative cost of flight time and connection priority the airline has shared, to judge which clearances the aircraft can fly and what each costs.</t>
         </is>
       </c>
-      <c r="G27" s="13" t="n"/>
+      <c r="G27" s="14" t="n"/>
+      <c r="H27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="15" t="n"/>
@@ -1301,7 +1359,8 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1330,7 +1389,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n"/>
+      <c r="G29" s="20" t="inlineStr">
+        <is>
+          <t>(no objective row)</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1344,6 +1408,7 @@
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
       <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1377,7 +1442,12 @@
           <t>The dispatcher shall file each flight's plan with air traffic control before departure.</t>
         </is>
       </c>
-      <c r="G31" s="13" t="n"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Flight Safety, Safety/separation</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n"/>
@@ -1404,7 +1474,8 @@
 (also comes from SLR-EXE-02)</t>
         </is>
       </c>
-      <c r="G32" s="13" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n"/>
@@ -1422,7 +1493,8 @@
 (also comes from SLR-CLR-10)</t>
         </is>
       </c>
-      <c r="G33" s="13" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="13" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="14" t="n"/>
@@ -1440,7 +1512,8 @@
 (also comes from SLR-CLR-02)</t>
         </is>
       </c>
-      <c r="G34" s="13" t="n"/>
+      <c r="G34" s="14" t="n"/>
+      <c r="H34" s="13" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="n"/>
@@ -1466,7 +1539,8 @@
           <t>ATC decision support shall alert the sector controller to each predicted loss of separation before it occurs.</t>
         </is>
       </c>
-      <c r="G35" s="13" t="n"/>
+      <c r="G35" s="14" t="n"/>
+      <c r="H35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="14" t="n"/>
@@ -1484,7 +1558,8 @@
 (also comes from SLR-CLR-01)</t>
         </is>
       </c>
-      <c r="G36" s="13" t="n"/>
+      <c r="G36" s="14" t="n"/>
+      <c r="H36" s="13" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="14" t="n"/>
@@ -1506,7 +1581,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G37" s="13" t="n"/>
+      <c r="G37" s="14" t="n"/>
+      <c r="H37" s="13" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="14" t="n"/>
@@ -1528,7 +1604,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G38" s="13" t="n"/>
+      <c r="G38" s="14" t="n"/>
+      <c r="H38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="n"/>
@@ -1554,7 +1631,8 @@
           <t>The en-route center shall inform the sector controller of each aircraft's filed route, requested altitude and requested speed before the aircraft enters the sector.</t>
         </is>
       </c>
-      <c r="G39" s="13" t="n"/>
+      <c r="G39" s="14" t="n"/>
+      <c r="H39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="n"/>
@@ -1581,7 +1659,8 @@
 (also comes from SLR-CLR-08, SLR-PLN-05)</t>
         </is>
       </c>
-      <c r="G40" s="13" t="n"/>
+      <c r="G40" s="14" t="n"/>
+      <c r="H40" s="13" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="14" t="n"/>
@@ -1599,7 +1678,8 @@
 (also comes from SLR-CLR-01)</t>
         </is>
       </c>
-      <c r="G41" s="13" t="n"/>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="13" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n"/>
@@ -1616,7 +1696,8 @@
           <t>The auto flight control system shall hold the aircraft on its cleared route, altitude and speed within the tolerances of the airspace.</t>
         </is>
       </c>
-      <c r="G42" s="13" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="13" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -1650,7 +1731,12 @@
           <t>The dispatcher shall file each flight's plan with air traffic control before departure.</t>
         </is>
       </c>
-      <c r="G43" s="13" t="n"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="14" t="n"/>
@@ -1672,7 +1758,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G44" s="13" t="n"/>
+      <c r="G44" s="14" t="n"/>
+      <c r="H44" s="13" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="14" t="n"/>
@@ -1694,7 +1781,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G45" s="13" t="n"/>
+      <c r="G45" s="14" t="n"/>
+      <c r="H45" s="13" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="15" t="n"/>
@@ -1716,7 +1804,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G46" s="13" t="n"/>
+      <c r="G46" s="15" t="n"/>
+      <c r="H46" s="13" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -1750,7 +1839,12 @@
           <t>The dispatcher shall file each flight's plan with air traffic control before departure.</t>
         </is>
       </c>
-      <c r="G47" s="13" t="n"/>
+      <c r="G47" s="16" t="inlineStr">
+        <is>
+          <t>Predictability</t>
+        </is>
+      </c>
+      <c r="H47" s="13" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="14" t="n"/>
@@ -1772,7 +1866,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G48" s="13" t="n"/>
+      <c r="G48" s="14" t="n"/>
+      <c r="H48" s="13" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="14" t="n"/>
@@ -1794,7 +1889,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G49" s="13" t="n"/>
+      <c r="G49" s="14" t="n"/>
+      <c r="H49" s="13" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="14" t="n"/>
@@ -1820,7 +1916,8 @@
           <t>The en-route center shall inform the sector controller of each aircraft's filed route, requested altitude and requested speed before the aircraft enters the sector.</t>
         </is>
       </c>
-      <c r="G50" s="13" t="n"/>
+      <c r="G50" s="14" t="n"/>
+      <c r="H50" s="13" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="14" t="n"/>
@@ -1841,7 +1938,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G51" s="13" t="n"/>
+      <c r="G51" s="14" t="n"/>
+      <c r="H51" s="13" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="14" t="n"/>
@@ -1868,7 +1966,8 @@
 (also comes from SLR-CLR-08, SLR-PLN-05)</t>
         </is>
       </c>
-      <c r="G52" s="13" t="n"/>
+      <c r="G52" s="14" t="n"/>
+      <c r="H52" s="13" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="14" t="n"/>
@@ -1886,7 +1985,8 @@
 (also comes from SLR-CLR-01)</t>
         </is>
       </c>
-      <c r="G53" s="13" t="n"/>
+      <c r="G53" s="14" t="n"/>
+      <c r="H53" s="13" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="15" t="n"/>
@@ -1903,7 +2003,8 @@
           <t>The auto flight control system shall hold the aircraft on its cleared route, altitude and speed within the tolerances of the airspace.</t>
         </is>
       </c>
-      <c r="G54" s="13" t="n"/>
+      <c r="G54" s="15" t="n"/>
+      <c r="H54" s="13" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -1936,7 +2037,12 @@
           <t>Air traffic control shall resolve each predicted conflict within the number of instructions the sector team can sustain.</t>
         </is>
       </c>
-      <c r="G55" s="13" t="n"/>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>Sector workload, Traffic complexity</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -1965,7 +2071,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G56" s="13" t="n"/>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>Delay (ATC-attributed)</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="15" t="n"/>
@@ -1986,7 +2097,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G57" s="13" t="n"/>
+      <c r="G57" s="15" t="n"/>
+      <c r="H57" s="13" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -2000,6 +2112,7 @@
       <c r="E58" s="6" t="n"/>
       <c r="F58" s="6" t="n"/>
       <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -2034,7 +2147,12 @@
 (also comes from SLR-EXE-02, SLR-CLR-08)</t>
         </is>
       </c>
-      <c r="G59" s="13" t="n"/>
+      <c r="G59" s="16" t="inlineStr">
+        <is>
+          <t>Safety, Operational flexibility</t>
+        </is>
+      </c>
+      <c r="H59" s="13" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="14" t="n"/>
@@ -2051,7 +2169,8 @@
           <t>The dispatcher shall release a flight only with the captain's agreement that it can be flown safely as planned.</t>
         </is>
       </c>
-      <c r="G60" s="13" t="n"/>
+      <c r="G60" s="14" t="n"/>
+      <c r="H60" s="13" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="14" t="n"/>
@@ -2078,7 +2197,8 @@
 (also comes from SLR-EXE-02, SLR-PLN-05)</t>
         </is>
       </c>
-      <c r="G61" s="13" t="n"/>
+      <c r="G61" s="14" t="n"/>
+      <c r="H61" s="13" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="15" t="n"/>
@@ -2100,7 +2220,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G62" s="13" t="n"/>
+      <c r="G62" s="15" t="n"/>
+      <c r="H62" s="13" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -2135,7 +2256,12 @@
 (also comes from SLR-PLN-02, SLR-PLN-04)</t>
         </is>
       </c>
-      <c r="G63" s="13" t="n"/>
+      <c r="G63" s="16" t="inlineStr">
+        <is>
+          <t>Safety, Procedural compliance</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="n"/>
@@ -2162,7 +2288,8 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G64" s="13" t="n"/>
+      <c r="G64" s="14" t="n"/>
+      <c r="H64" s="13" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="n"/>
@@ -2179,7 +2306,8 @@
           <t>Flight operations shall give the flight crew the dispatch release, flight plan, weather, notices to airmen (NOTAMs) and load sheet before departure.</t>
         </is>
       </c>
-      <c r="G65" s="13" t="n"/>
+      <c r="G65" s="14" t="n"/>
+      <c r="H65" s="13" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="n"/>
@@ -2197,7 +2325,8 @@
 (also comes from SLR-APT-04)</t>
         </is>
       </c>
-      <c r="G66" s="13" t="n"/>
+      <c r="G66" s="14" t="n"/>
+      <c r="H66" s="13" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n"/>
@@ -2219,7 +2348,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G67" s="13" t="n"/>
+      <c r="G67" s="14" t="n"/>
+      <c r="H67" s="13" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n"/>
@@ -2246,7 +2376,8 @@
 (also comes from SLR-INF-07, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G68" s="13" t="n"/>
+      <c r="G68" s="14" t="n"/>
+      <c r="H68" s="13" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="14" t="n"/>
@@ -2264,7 +2395,8 @@
 (also comes from SLR-CLR-04, SLR-INF-07)</t>
         </is>
       </c>
-      <c r="G69" s="13" t="n"/>
+      <c r="G69" s="14" t="n"/>
+      <c r="H69" s="13" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="15" t="n"/>
@@ -2281,7 +2413,8 @@
           <t>The flight management system shall alert the flight crew when the fuel it predicts at the destination falls below the required reserve.</t>
         </is>
       </c>
-      <c r="G70" s="13" t="n"/>
+      <c r="G70" s="15" t="n"/>
+      <c r="H70" s="13" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -2314,7 +2447,12 @@
           <t>The flight crew shall accept a clearance only if the aircraft can fly it, and shall answer 'unable' when it cannot.</t>
         </is>
       </c>
-      <c r="G71" s="13" t="n"/>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>Safety, Workload</t>
+        </is>
+      </c>
+      <c r="H71" s="13" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="14" t="n"/>
@@ -2332,7 +2470,8 @@
 (also comes from SLR-CLR-01)</t>
         </is>
       </c>
-      <c r="G72" s="13" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="13" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="n"/>
@@ -2358,7 +2497,8 @@
           <t>[IMPROVED] Flight operations shall make each flight's current gross weight, performance model, relative cost of flight time and connection priority available to the party that decides a change to that flight's trajectory.</t>
         </is>
       </c>
-      <c r="G73" s="13" t="n"/>
+      <c r="G73" s="14" t="n"/>
+      <c r="H73" s="13" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="14" t="n"/>
@@ -2375,7 +2515,8 @@
           <t>[IMPROVED] ATC decision support shall use the best information available to it about each flight, including the gross weight, performance model, relative cost of flight time and connection priority the airline has shared, to judge which clearances the aircraft can fly and what each costs.</t>
         </is>
       </c>
-      <c r="G74" s="13" t="n"/>
+      <c r="G74" s="14" t="n"/>
+      <c r="H74" s="13" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="14" t="n"/>
@@ -2393,7 +2534,8 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G75" s="13" t="n"/>
+      <c r="G75" s="14" t="n"/>
+      <c r="H75" s="13" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="14" t="n"/>
@@ -2420,7 +2562,8 @@
 (also comes from SLR-CLR-09)</t>
         </is>
       </c>
-      <c r="G76" s="13" t="n"/>
+      <c r="G76" s="14" t="n"/>
+      <c r="H76" s="13" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="14" t="n"/>
@@ -2438,7 +2581,8 @@
 (also comes from SLR-PLN-07)</t>
         </is>
       </c>
-      <c r="G77" s="13" t="n"/>
+      <c r="G77" s="14" t="n"/>
+      <c r="H77" s="13" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="14" t="n"/>
@@ -2455,7 +2599,8 @@
           <t>The flight management system shall predict the flight's arrival time, fuel at the destination, optimum altitude and maximum altitude from the entered weights, the cost index and the forecast winds.</t>
         </is>
       </c>
-      <c r="G78" s="13" t="n"/>
+      <c r="G78" s="14" t="n"/>
+      <c r="H78" s="13" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="14" t="n"/>
@@ -2473,7 +2618,8 @@
 (also comes from SLR-INF-02)</t>
         </is>
       </c>
-      <c r="G79" s="13" t="n"/>
+      <c r="G79" s="14" t="n"/>
+      <c r="H79" s="13" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="14" t="n"/>
@@ -2500,7 +2646,8 @@
 (also comes from SLR-INF-07, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G80" s="13" t="n"/>
+      <c r="G80" s="14" t="n"/>
+      <c r="H80" s="13" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="14" t="n"/>
@@ -2518,7 +2665,8 @@
 (also comes from SLR-CLR-04, SLR-INF-07)</t>
         </is>
       </c>
-      <c r="G81" s="13" t="n"/>
+      <c r="G81" s="14" t="n"/>
+      <c r="H81" s="13" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="15" t="n"/>
@@ -2535,7 +2683,8 @@
           <t>The flight management system shall alert the flight crew when the fuel it predicts at the destination falls below the required reserve.</t>
         </is>
       </c>
-      <c r="G82" s="13" t="n"/>
+      <c r="G82" s="15" t="n"/>
+      <c r="H82" s="13" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -2570,7 +2719,12 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G83" s="13" t="n"/>
+      <c r="G83" s="16" t="inlineStr">
+        <is>
+          <t>Operational flexibility</t>
+        </is>
+      </c>
+      <c r="H83" s="13" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="15" t="n"/>
@@ -2587,7 +2741,8 @@
           <t>Air traffic control shall answer each flight crew request for a route, altitude or speed change with an approval, an amended clearance or 'unable'.</t>
         </is>
       </c>
-      <c r="G84" s="13" t="n"/>
+      <c r="G84" s="15" t="n"/>
+      <c r="H84" s="13" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -2617,7 +2772,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G85" s="13" t="n"/>
+      <c r="G85" s="16" t="inlineStr">
+        <is>
+          <t>Schedule/duty constraints</t>
+        </is>
+      </c>
+      <c r="H85" s="13" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -2652,7 +2812,12 @@
 (also comes from SLR-EXE-02)</t>
         </is>
       </c>
-      <c r="G86" s="13" t="n"/>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="H86" s="13" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="14" t="n"/>
@@ -2670,7 +2835,8 @@
 (also comes from SLR-CLR-10)</t>
         </is>
       </c>
-      <c r="G87" s="13" t="n"/>
+      <c r="G87" s="14" t="n"/>
+      <c r="H87" s="13" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="14" t="n"/>
@@ -2688,7 +2854,8 @@
 (also comes from SLR-CLR-02)</t>
         </is>
       </c>
-      <c r="G88" s="13" t="n"/>
+      <c r="G88" s="14" t="n"/>
+      <c r="H88" s="13" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="14" t="n"/>
@@ -2714,7 +2881,8 @@
           <t>ATC decision support shall alert the sector controller to each predicted loss of separation before it occurs.</t>
         </is>
       </c>
-      <c r="G89" s="13" t="n"/>
+      <c r="G89" s="14" t="n"/>
+      <c r="H89" s="13" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="15" t="n"/>
@@ -2732,7 +2900,8 @@
 (also comes from SLR-CLR-01)</t>
         </is>
       </c>
-      <c r="G90" s="13" t="n"/>
+      <c r="G90" s="15" t="n"/>
+      <c r="H90" s="13" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -2767,7 +2936,12 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G91" s="13" t="n"/>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>Safety, Procedural compliance</t>
+        </is>
+      </c>
+      <c r="H91" s="13" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="14" t="n"/>
@@ -2784,7 +2958,8 @@
           <t>Flight operations shall give the flight crew the dispatch release, flight plan, weather, notices to airmen (NOTAMs) and load sheet before departure.</t>
         </is>
       </c>
-      <c r="G92" s="13" t="n"/>
+      <c r="G92" s="14" t="n"/>
+      <c r="H92" s="13" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="15" t="n"/>
@@ -2802,7 +2977,8 @@
 (also comes from SLR-APT-04)</t>
         </is>
       </c>
-      <c r="G93" s="13" t="n"/>
+      <c r="G93" s="15" t="n"/>
+      <c r="H93" s="13" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -2837,7 +3013,12 @@
 (also comes from SLR-INF-07, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G94" s="13" t="n"/>
+      <c r="G94" s="8" t="inlineStr">
+        <is>
+          <t>Workload, Procedural compliance</t>
+        </is>
+      </c>
+      <c r="H94" s="13" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="14" t="n"/>
@@ -2855,7 +3036,8 @@
 (also comes from SLR-INF-07, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G95" s="13" t="n"/>
+      <c r="G95" s="14" t="n"/>
+      <c r="H95" s="13" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="15" t="n"/>
@@ -2872,7 +3054,8 @@
           <t>The aircraft communication system shall carry voice and data between the flight crew and both air traffic control and the dispatcher for the whole flight.</t>
         </is>
       </c>
-      <c r="G96" s="13" t="n"/>
+      <c r="G96" s="15" t="n"/>
+      <c r="H96" s="13" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -2886,6 +3069,7 @@
       <c r="E97" s="6" t="n"/>
       <c r="F97" s="6" t="n"/>
       <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -2893,7 +3077,7 @@
           <t>SN-GOV-01</t>
         </is>
       </c>
-      <c r="B98" s="20" t="inlineStr">
+      <c r="B98" s="21" t="inlineStr">
         <is>
           <t>[BACKGROUND] The NAS shall conduct every flight within the operating rules of 14 CFR and the FAA's air traffic orders.</t>
         </is>
@@ -2920,7 +3104,12 @@
 (also comes from SLR-PLN-01, SLR-PLN-02)</t>
         </is>
       </c>
-      <c r="G98" s="13" t="n"/>
+      <c r="G98" s="22" t="inlineStr">
+        <is>
+          <t>(no objective row)</t>
+        </is>
+      </c>
+      <c r="H98" s="13" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="14" t="n"/>
@@ -2947,7 +3136,8 @@
 (also comes from SLR-EXE-02, SLR-CLR-08)</t>
         </is>
       </c>
-      <c r="G99" s="13" t="n"/>
+      <c r="G99" s="14" t="n"/>
+      <c r="H99" s="13" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="14" t="n"/>
@@ -2964,7 +3154,8 @@
           <t>The dispatcher shall release a flight only with the captain's agreement that it can be flown safely as planned.</t>
         </is>
       </c>
-      <c r="G100" s="13" t="n"/>
+      <c r="G100" s="14" t="n"/>
+      <c r="H100" s="13" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="14" t="n"/>
@@ -2986,7 +3177,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G101" s="13" t="n"/>
+      <c r="G101" s="14" t="n"/>
+      <c r="H101" s="13" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="14" t="n"/>
@@ -3013,7 +3205,8 @@
 (also comes from SLR-EXE-02, SLR-PLN-05)</t>
         </is>
       </c>
-      <c r="G102" s="13" t="n"/>
+      <c r="G102" s="14" t="n"/>
+      <c r="H102" s="13" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="14" t="n"/>
@@ -3040,7 +3233,8 @@
 (also comes from SLR-INF-07, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G103" s="13" t="n"/>
+      <c r="G103" s="14" t="n"/>
+      <c r="H103" s="13" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="14" t="n"/>
@@ -3058,7 +3252,8 @@
 (also comes from SLR-CLR-04, SLR-INF-07)</t>
         </is>
       </c>
-      <c r="G104" s="13" t="n"/>
+      <c r="G104" s="14" t="n"/>
+      <c r="H104" s="13" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="14" t="n"/>
@@ -3075,7 +3270,8 @@
           <t>The flight management system shall alert the flight crew when the fuel it predicts at the destination falls below the required reserve.</t>
         </is>
       </c>
-      <c r="G105" s="13" t="n"/>
+      <c r="G105" s="14" t="n"/>
+      <c r="H105" s="13" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="15" t="n"/>
@@ -3101,7 +3297,8 @@
           <t>Air traffic control shall record each clearance it issues with the issuing facility and the time.</t>
         </is>
       </c>
-      <c r="G106" s="13" t="n"/>
+      <c r="G106" s="15" t="n"/>
+      <c r="H106" s="13" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -3136,7 +3333,12 @@
 (also comes from SLR-EXE-02, SLR-CLR-08)</t>
         </is>
       </c>
-      <c r="G107" s="13" t="n"/>
+      <c r="G107" s="20" t="inlineStr">
+        <is>
+          <t>(no objective row)</t>
+        </is>
+      </c>
+      <c r="H107" s="13" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="14" t="n"/>
@@ -3153,7 +3355,8 @@
           <t>The dispatcher shall release a flight only with the captain's agreement that it can be flown safely as planned.</t>
         </is>
       </c>
-      <c r="G108" s="13" t="n"/>
+      <c r="G108" s="14" t="n"/>
+      <c r="H108" s="13" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="14" t="n"/>
@@ -3175,7 +3378,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G109" s="13" t="n"/>
+      <c r="G109" s="14" t="n"/>
+      <c r="H109" s="13" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="14" t="n"/>
@@ -3197,7 +3401,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G110" s="13" t="n"/>
+      <c r="G110" s="14" t="n"/>
+      <c r="H110" s="13" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="15" t="n"/>
@@ -3223,7 +3428,8 @@
           <t>Air traffic control shall record each clearance it issues with the issuing facility and the time.</t>
         </is>
       </c>
-      <c r="G111" s="13" t="n"/>
+      <c r="G111" s="15" t="n"/>
+      <c r="H111" s="13" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -3237,6 +3443,7 @@
       <c r="E112" s="6" t="n"/>
       <c r="F112" s="6" t="n"/>
       <c r="G112" s="6" t="n"/>
+      <c r="H112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -3244,7 +3451,7 @@
           <t>SN-ENV-01</t>
         </is>
       </c>
-      <c r="B113" s="20" t="inlineStr">
+      <c r="B113" s="21" t="inlineStr">
         <is>
           <t>[BACKGROUND] The NAS shall keep the CO2 emitted by each flight as low as safety, economics and capacity allow.</t>
         </is>
@@ -3270,7 +3477,12 @@
           <t>[GOAL, IMPROVED] Air traffic control should choose, among the clearances that resolve a conflict and can be flown, the one with the lowest impact on the systems involved.</t>
         </is>
       </c>
-      <c r="G113" s="13" t="n"/>
+      <c r="G113" s="21" t="inlineStr">
+        <is>
+          <t>CO2, NOx, Contrail/climate effects, Local air quality</t>
+        </is>
+      </c>
+      <c r="H113" s="13" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="14" t="n"/>
@@ -3292,7 +3504,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G114" s="13" t="n"/>
+      <c r="G114" s="14" t="n"/>
+      <c r="H114" s="13" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="15" t="n"/>
@@ -3318,7 +3531,8 @@
           <t>Flight operations shall report each flight's fuel burned and its CO2 emitted at 3.16 kg of CO2 per kg of fuel.</t>
         </is>
       </c>
-      <c r="G115" s="13" t="n"/>
+      <c r="G115" s="15" t="n"/>
+      <c r="H115" s="13" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -3347,7 +3561,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G116" s="13" t="n"/>
+      <c r="G116" s="16" t="inlineStr">
+        <is>
+          <t>Noise</t>
+        </is>
+      </c>
+      <c r="H116" s="13" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
@@ -3361,6 +3580,7 @@
       <c r="E117" s="6" t="n"/>
       <c r="F117" s="6" t="n"/>
       <c r="G117" s="6" t="n"/>
+      <c r="H117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -3395,7 +3615,12 @@
 (also comes from SLR-EXE-06, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G118" s="13" t="n"/>
+      <c r="G118" s="16" t="inlineStr">
+        <is>
+          <t>Gate utilization, Turnaround performance, Passenger throughput</t>
+        </is>
+      </c>
+      <c r="H118" s="13" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="14" t="n"/>
@@ -3413,7 +3638,8 @@
 (also comes from SLR-CLR-04, SLR-EXE-06)</t>
         </is>
       </c>
-      <c r="G119" s="13" t="n"/>
+      <c r="G119" s="14" t="n"/>
+      <c r="H119" s="13" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="15" t="n"/>
@@ -3435,7 +3661,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G120" s="13" t="n"/>
+      <c r="G120" s="15" t="n"/>
+      <c r="H120" s="13" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -3465,7 +3692,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G121" s="13" t="n"/>
+      <c r="G121" s="16" t="inlineStr">
+        <is>
+          <t>Runway utilization</t>
+        </is>
+      </c>
+      <c r="H121" s="13" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -3495,7 +3727,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G122" s="13" t="n"/>
+      <c r="G122" s="16" t="inlineStr">
+        <is>
+          <t>Surface congestion</t>
+        </is>
+      </c>
+      <c r="H122" s="13" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
@@ -3509,6 +3746,7 @@
       <c r="E123" s="6" t="n"/>
       <c r="F123" s="6" t="n"/>
       <c r="G123" s="6" t="n"/>
+      <c r="H123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -3543,7 +3781,12 @@
 (also comes from SLR-PLN-01, SLR-PLN-02)</t>
         </is>
       </c>
-      <c r="G124" s="13" t="n"/>
+      <c r="G124" s="16" t="inlineStr">
+        <is>
+          <t>Flight Safety</t>
+        </is>
+      </c>
+      <c r="H124" s="13" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="14" t="n"/>
@@ -3570,7 +3813,8 @@
 (also comes from SLR-EXE-02)</t>
         </is>
       </c>
-      <c r="G125" s="13" t="n"/>
+      <c r="G125" s="14" t="n"/>
+      <c r="H125" s="13" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="14" t="n"/>
@@ -3588,7 +3832,8 @@
 (also comes from SLR-CLR-10)</t>
         </is>
       </c>
-      <c r="G126" s="13" t="n"/>
+      <c r="G126" s="14" t="n"/>
+      <c r="H126" s="13" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="14" t="n"/>
@@ -3606,7 +3851,8 @@
 (also comes from SLR-CLR-02)</t>
         </is>
       </c>
-      <c r="G127" s="13" t="n"/>
+      <c r="G127" s="14" t="n"/>
+      <c r="H127" s="13" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="14" t="n"/>
@@ -3633,7 +3879,8 @@
 (also comes from SLR-EXE-02, SLR-PLN-05)</t>
         </is>
       </c>
-      <c r="G128" s="13" t="n"/>
+      <c r="G128" s="14" t="n"/>
+      <c r="H128" s="13" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="14" t="n"/>
@@ -3660,7 +3907,8 @@
 (also comes from SLR-INF-07, SLR-CLR-04)</t>
         </is>
       </c>
-      <c r="G129" s="13" t="n"/>
+      <c r="G129" s="14" t="n"/>
+      <c r="H129" s="13" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="14" t="n"/>
@@ -3678,7 +3926,8 @@
 (also comes from SLR-CLR-04, SLR-INF-07)</t>
         </is>
       </c>
-      <c r="G130" s="13" t="n"/>
+      <c r="G130" s="14" t="n"/>
+      <c r="H130" s="13" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="15" t="n"/>
@@ -3695,7 +3944,8 @@
           <t>The flight management system shall alert the flight crew when the fuel it predicts at the destination falls below the required reserve.</t>
         </is>
       </c>
-      <c r="G131" s="13" t="n"/>
+      <c r="G131" s="15" t="n"/>
+      <c r="H131" s="13" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -3725,7 +3975,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G132" s="13" t="n"/>
+      <c r="G132" s="16" t="inlineStr">
+        <is>
+          <t>Travel time, Connection reliability, Disruption risk</t>
+        </is>
+      </c>
+      <c r="H132" s="13" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -3760,7 +4015,12 @@
 (also comes from SLR-EXE-03)</t>
         </is>
       </c>
-      <c r="G133" s="13" t="n"/>
+      <c r="G133" s="16" t="inlineStr">
+        <is>
+          <t>Comfort</t>
+        </is>
+      </c>
+      <c r="H133" s="13" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="14" t="n"/>
@@ -3777,7 +4037,8 @@
           <t>Air traffic control shall answer each flight crew request for a route, altitude or speed change with an approval, an amended clearance or 'unable'.</t>
         </is>
       </c>
-      <c r="G134" s="13" t="n"/>
+      <c r="G134" s="14" t="n"/>
+      <c r="H134" s="13" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="15" t="n"/>
@@ -3799,7 +4060,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G135" s="13" t="n"/>
+      <c r="G135" s="15" t="n"/>
+      <c r="H135" s="13" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
@@ -3813,6 +4075,7 @@
       <c r="E136" s="6" t="n"/>
       <c r="F136" s="6" t="n"/>
       <c r="G136" s="6" t="n"/>
+      <c r="H136" s="6" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -3842,7 +4105,12 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G137" s="13" t="n"/>
+      <c r="G137" s="16" t="inlineStr">
+        <is>
+          <t>Airspace access</t>
+        </is>
+      </c>
+      <c r="H137" s="13" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="14" t="n"/>
@@ -3864,7 +4132,8 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G138" s="13" t="n"/>
+      <c r="G138" s="14" t="n"/>
+      <c r="H138" s="13" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="15" t="n"/>
@@ -3885,11 +4154,14 @@
           <t>(no HLR: not carried into the study)</t>
         </is>
       </c>
-      <c r="G139" s="13" t="n"/>
+      <c r="G139" s="15" t="n"/>
+      <c r="H139" s="13" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G139"/>
-  <mergeCells count="104">
+  <autoFilter ref="A1:H139"/>
+  <mergeCells count="126">
+    <mergeCell ref="G3:G11"/>
+    <mergeCell ref="G12:G17"/>
     <mergeCell ref="D99:D100"/>
     <mergeCell ref="A3:A11"/>
     <mergeCell ref="B59:B62"/>
@@ -3905,11 +4177,17 @@
     <mergeCell ref="C73:C75"/>
     <mergeCell ref="A107:A111"/>
     <mergeCell ref="D80:D82"/>
+    <mergeCell ref="G25:G28"/>
     <mergeCell ref="B86:B90"/>
     <mergeCell ref="B56:B57"/>
     <mergeCell ref="C52:C54"/>
     <mergeCell ref="A133:A135"/>
+    <mergeCell ref="G59:G62"/>
+    <mergeCell ref="G63:G70"/>
     <mergeCell ref="A86:A90"/>
+    <mergeCell ref="G43:G46"/>
+    <mergeCell ref="G133:G135"/>
+    <mergeCell ref="G94:G96"/>
     <mergeCell ref="A31:A42"/>
     <mergeCell ref="B18:B23"/>
     <mergeCell ref="B43:B46"/>
@@ -3921,6 +4199,7 @@
     <mergeCell ref="B71:B82"/>
     <mergeCell ref="A12:A17"/>
     <mergeCell ref="D118:D119"/>
+    <mergeCell ref="G86:G90"/>
     <mergeCell ref="C64:C66"/>
     <mergeCell ref="C7:C10"/>
     <mergeCell ref="A137:A139"/>
@@ -3932,6 +4211,7 @@
     <mergeCell ref="D86:D88"/>
     <mergeCell ref="B3:B11"/>
     <mergeCell ref="C83:C84"/>
+    <mergeCell ref="G137:G139"/>
     <mergeCell ref="D32:D34"/>
     <mergeCell ref="C107:C108"/>
     <mergeCell ref="D103:D105"/>
@@ -3942,7 +4222,10 @@
     <mergeCell ref="C59:C60"/>
     <mergeCell ref="C22:C23"/>
     <mergeCell ref="D129:D131"/>
+    <mergeCell ref="G31:G42"/>
     <mergeCell ref="A63:A70"/>
+    <mergeCell ref="G98:G106"/>
+    <mergeCell ref="G71:G82"/>
     <mergeCell ref="D73:D75"/>
     <mergeCell ref="B113:B115"/>
     <mergeCell ref="C12:C13"/>
@@ -3953,18 +4236,22 @@
     <mergeCell ref="D107:D108"/>
     <mergeCell ref="B91:B93"/>
     <mergeCell ref="B83:B84"/>
+    <mergeCell ref="G124:G131"/>
     <mergeCell ref="D83:D84"/>
     <mergeCell ref="D52:D54"/>
     <mergeCell ref="C94:C96"/>
     <mergeCell ref="D133:D134"/>
+    <mergeCell ref="G56:G57"/>
     <mergeCell ref="A43:A46"/>
     <mergeCell ref="D91:D93"/>
     <mergeCell ref="A83:A84"/>
     <mergeCell ref="A71:A82"/>
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="A113:A115"/>
+    <mergeCell ref="G47:G54"/>
     <mergeCell ref="C89:C90"/>
     <mergeCell ref="A91:A93"/>
+    <mergeCell ref="G113:G115"/>
     <mergeCell ref="B98:B106"/>
     <mergeCell ref="C91:C93"/>
     <mergeCell ref="D64:D66"/>
@@ -3974,14 +4261,18 @@
     <mergeCell ref="C118:C119"/>
     <mergeCell ref="C133:C134"/>
     <mergeCell ref="B12:B17"/>
+    <mergeCell ref="G91:G93"/>
+    <mergeCell ref="G83:G84"/>
     <mergeCell ref="C99:C100"/>
     <mergeCell ref="C19:C21"/>
     <mergeCell ref="D7:D10"/>
+    <mergeCell ref="G18:G23"/>
     <mergeCell ref="A124:A131"/>
     <mergeCell ref="D40:D42"/>
     <mergeCell ref="A18:A23"/>
     <mergeCell ref="A94:A96"/>
     <mergeCell ref="C103:C105"/>
+    <mergeCell ref="G107:G111"/>
     <mergeCell ref="D89:D90"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="A118:A120"/>
@@ -3991,6 +4282,7 @@
     <mergeCell ref="C80:C82"/>
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="C129:C131"/>
+    <mergeCell ref="G118:G120"/>
     <mergeCell ref="B137:B139"/>
     <mergeCell ref="D59:D60"/>
     <mergeCell ref="D22:D23"/>
@@ -4121,7 +4413,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>GAP: stakeholder requirement with no system requirement</t>
         </is>
@@ -4132,7 +4424,7 @@
       <c r="C8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>GAP: system requirement with no stakeholder parent</t>
         </is>
@@ -4143,7 +4435,7 @@
       <c r="C9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>GAP: system requirement in the study with no HLR</t>
         </is>
@@ -4154,7 +4446,7 @@
       <c r="C10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>GAP: system requirement with no allocation</t>
         </is>
@@ -4165,7 +4457,7 @@
       <c r="C11" s="13" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>GAP: HLR with no allocation</t>
         </is>
@@ -4176,7 +4468,7 @@
       <c r="C12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>CHECK: out-of-study system requirement that has an HLR</t>
         </is>
@@ -4187,7 +4479,7 @@
       <c r="C13" s="13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>CHECK: in-study system requirement whose only parents are out of study</t>
         </is>
@@ -4198,7 +4490,7 @@
       <c r="C14" s="13" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>CHECK: HLR reached only through out-of-study system requirements</t>
         </is>
@@ -4280,7 +4572,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Fuel cost</t>
         </is>
@@ -4314,7 +4606,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>Crew cost</t>
         </is>
@@ -4348,7 +4640,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>Aircraft utilization</t>
         </is>
@@ -4382,7 +4674,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>Maintenance</t>
         </is>
@@ -4416,7 +4708,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Schedule integrity</t>
         </is>
@@ -4450,7 +4742,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>Passenger connections</t>
         </is>
@@ -4488,7 +4780,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Delay cost</t>
         </is>
@@ -4526,7 +4818,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
@@ -4560,7 +4852,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Dispatch reliability</t>
         </is>
@@ -4594,7 +4886,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>Flight Safety</t>
         </is>
@@ -4632,7 +4924,7 @@
           <t>Passenger</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Ticket price</t>
         </is>
@@ -4666,7 +4958,7 @@
           <t>Passenger</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Travel time</t>
         </is>
@@ -4704,7 +4996,7 @@
           <t>Passenger</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Connection reliability</t>
         </is>
@@ -4742,7 +5034,7 @@
           <t>Passenger</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>Schedule convenience</t>
         </is>
@@ -4776,7 +5068,7 @@
           <t>Passenger</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>Comfort</t>
         </is>
@@ -4814,7 +5106,7 @@
           <t>Passenger</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>Disruption risk</t>
         </is>
@@ -4852,7 +5144,7 @@
           <t>ATC / ANSP</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>Safety/separation</t>
         </is>
@@ -4886,7 +5178,7 @@
           <t>ATC / ANSP</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>Sector workload</t>
         </is>
@@ -4920,7 +5212,7 @@
           <t>ATC / ANSP</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
@@ -4954,7 +5246,7 @@
           <t>ATC / ANSP</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>Predictability</t>
         </is>
@@ -4992,7 +5284,7 @@
           <t>ATC / ANSP</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="23" t="inlineStr">
         <is>
           <t>Delay (ATC-attributed)</t>
         </is>
@@ -5030,7 +5322,7 @@
           <t>ATC / ANSP</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>Traffic complexity</t>
         </is>
@@ -5064,7 +5356,7 @@
           <t>Airport</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>Gate utilization</t>
         </is>
@@ -5102,7 +5394,7 @@
           <t>Airport</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>Runway utilization</t>
         </is>
@@ -5140,7 +5432,7 @@
           <t>Airport</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
         <is>
           <t>Surface congestion</t>
         </is>
@@ -5178,7 +5470,7 @@
           <t>Airport</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>Turnaround performance</t>
         </is>
@@ -5216,7 +5508,7 @@
           <t>Airport</t>
         </is>
       </c>
-      <c r="B28" s="21" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>Passenger throughput</t>
         </is>
@@ -5254,7 +5546,7 @@
           <t>Flight Crew</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
@@ -5292,7 +5584,7 @@
           <t>Flight Crew</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>Workload</t>
         </is>
@@ -5326,7 +5618,7 @@
           <t>Flight Crew</t>
         </is>
       </c>
-      <c r="B31" s="21" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>Procedural compliance</t>
         </is>
@@ -5364,7 +5656,7 @@
           <t>Flight Crew</t>
         </is>
       </c>
-      <c r="B32" s="21" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>Schedule/duty constraints</t>
         </is>
@@ -5402,7 +5694,7 @@
           <t>Flight Crew</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Operational flexibility</t>
         </is>
@@ -5440,7 +5732,7 @@
           <t>Environmental / Societal</t>
         </is>
       </c>
-      <c r="B34" s="21" t="inlineStr">
+      <c r="B34" s="23" t="inlineStr">
         <is>
           <t>CO2</t>
         </is>
@@ -5478,7 +5770,7 @@
           <t>Environmental / Societal</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t>NOx</t>
         </is>
@@ -5516,7 +5808,7 @@
           <t>Environmental / Societal</t>
         </is>
       </c>
-      <c r="B36" s="21" t="inlineStr">
+      <c r="B36" s="23" t="inlineStr">
         <is>
           <t>Contrail/climate effects</t>
         </is>
@@ -5554,7 +5846,7 @@
           <t>Environmental / Societal</t>
         </is>
       </c>
-      <c r="B37" s="21" t="inlineStr">
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>Noise</t>
         </is>
@@ -5592,7 +5884,7 @@
           <t>Environmental / Societal</t>
         </is>
       </c>
-      <c r="B38" s="21" t="inlineStr">
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t>Local air quality</t>
         </is>
@@ -5703,29 +5995,29 @@
       <c r="H41" s="13" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>Military</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="24" t="inlineStr">
         <is>
           <t>Airspace access</t>
         </is>
       </c>
-      <c r="C42" s="22" t="inlineStr">
+      <c r="C42" s="24" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr"/>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="D42" s="24" t="inlineStr"/>
+      <c r="E42" s="24" t="inlineStr">
         <is>
           <t>SN-MIL-01 (out of study)</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr"/>
-      <c r="G42" s="22" t="inlineStr"/>
+      <c r="F42" s="24" t="inlineStr"/>
+      <c r="G42" s="24" t="inlineStr"/>
       <c r="H42" s="13" t="n"/>
     </row>
     <row r="43">
@@ -5786,7 +6078,7 @@
           <t>Airline</t>
         </is>
       </c>
-      <c r="B45" s="23" t="inlineStr">
+      <c r="B45" s="25" t="inlineStr">
         <is>
           <t>(no objective row)</t>
         </is>
@@ -5808,7 +6100,7 @@
           <t>Regulator</t>
         </is>
       </c>
-      <c r="B46" s="23" t="inlineStr">
+      <c r="B46" s="25" t="inlineStr">
         <is>
           <t>(no objective row)</t>
         </is>
@@ -5830,7 +6122,7 @@
           <t>Regulator</t>
         </is>
       </c>
-      <c r="B47" s="23" t="inlineStr">
+      <c r="B47" s="25" t="inlineStr">
         <is>
           <t>(no objective row)</t>
         </is>
@@ -5932,7 +6224,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>SN-AIR-01</t>
         </is>
@@ -5985,7 +6277,7 @@
       <c r="K2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>SN-AIR-02</t>
         </is>
@@ -6034,7 +6326,7 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>SN-AIR-03</t>
         </is>
@@ -6087,7 +6379,7 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>SN-AIR-04</t>
         </is>
@@ -6112,7 +6404,7 @@
           <t>SLR-FLW-04</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6140,7 +6432,7 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>SN-AIR-05</t>
         </is>
@@ -6193,7 +6485,7 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>SN-AIR-06</t>
         </is>
@@ -6218,7 +6510,7 @@
           <t>SLR-INF-05</t>
         </is>
       </c>
-      <c r="F7" s="22" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6246,7 +6538,7 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>SN-ATC-01</t>
         </is>
@@ -6299,7 +6591,7 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>SN-ATC-02</t>
         </is>
@@ -6352,7 +6644,7 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>SN-ATC-03</t>
         </is>
@@ -6377,7 +6669,7 @@
           <t>SLR-PLN-06, SLR-FLW-06, SLR-CLR-03, SLR-INF-01, SLR-EXE-01, SLR-EXE-02</t>
         </is>
       </c>
-      <c r="F10" s="22" t="inlineStr">
+      <c r="F10" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6405,7 +6697,7 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>SN-ATC-04</t>
         </is>
@@ -6458,7 +6750,7 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>SN-ATC-05</t>
         </is>
@@ -6483,7 +6775,7 @@
           <t>SLR-FLW-05, SLR-MEA-04</t>
         </is>
       </c>
-      <c r="F12" s="22" t="inlineStr">
+      <c r="F12" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6511,7 +6803,7 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-01</t>
         </is>
@@ -6536,7 +6828,7 @@
           <t>SLR-PLN-05, SLR-CLR-08, SLR-EXE-04</t>
         </is>
       </c>
-      <c r="F13" s="22" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6564,7 +6856,7 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-02</t>
         </is>
@@ -6589,7 +6881,7 @@
           <t>SLR-PLN-01, SLR-PLN-07, SLR-INF-06, SLR-EXE-06</t>
         </is>
       </c>
-      <c r="F14" s="22" t="inlineStr">
+      <c r="F14" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6617,7 +6909,7 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-03</t>
         </is>
@@ -6666,7 +6958,7 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-04</t>
         </is>
@@ -6691,7 +6983,7 @@
           <t>SLR-CLR-09</t>
         </is>
       </c>
-      <c r="F16" s="22" t="inlineStr">
+      <c r="F16" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6719,7 +7011,7 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-05</t>
         </is>
@@ -6744,7 +7036,7 @@
           <t>SLR-PLN-09</t>
         </is>
       </c>
-      <c r="F17" s="22" t="inlineStr">
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -6772,7 +7064,7 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-06</t>
         </is>
@@ -6821,7 +7113,7 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-07</t>
         </is>
@@ -6870,7 +7162,7 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>SN-CRW-08</t>
         </is>
@@ -6919,7 +7211,7 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>SN-GOV-01</t>
         </is>
@@ -6944,7 +7236,7 @@
           <t>SLR-PLN-04, SLR-PLN-05, SLR-PLN-09, SLR-CLR-08, SLR-EXE-06, SLR-MEA-01</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="21" t="inlineStr">
         <is>
           <t>background</t>
         </is>
@@ -6972,7 +7264,7 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>SN-GOV-02</t>
         </is>
@@ -6997,7 +7289,7 @@
           <t>SLR-PLN-05, SLR-CLR-05, SLR-EXE-04, SLR-MEA-01</t>
         </is>
       </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="F22" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7025,7 +7317,7 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>SN-ENV-01</t>
         </is>
@@ -7050,7 +7342,7 @@
           <t>SLR-CLR-13, SLR-APT-03, SLR-MEA-02</t>
         </is>
       </c>
-      <c r="F23" s="20" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>background</t>
         </is>
@@ -7078,7 +7370,7 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>SN-ENV-02</t>
         </is>
@@ -7103,7 +7395,7 @@
           <t>SLR-APT-05</t>
         </is>
       </c>
-      <c r="F24" s="22" t="inlineStr">
+      <c r="F24" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7127,7 +7419,7 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>SN-APT-01</t>
         </is>
@@ -7152,7 +7444,7 @@
           <t>SLR-INF-07, SLR-APT-01</t>
         </is>
       </c>
-      <c r="F25" s="22" t="inlineStr">
+      <c r="F25" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7176,7 +7468,7 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>SN-APT-02</t>
         </is>
@@ -7201,7 +7493,7 @@
           <t>SLR-APT-02</t>
         </is>
       </c>
-      <c r="F26" s="22" t="inlineStr">
+      <c r="F26" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7225,7 +7517,7 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>SN-APT-03</t>
         </is>
@@ -7250,7 +7542,7 @@
           <t>SLR-APT-03</t>
         </is>
       </c>
-      <c r="F27" s="22" t="inlineStr">
+      <c r="F27" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7274,7 +7566,7 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>SN-PAX-01</t>
         </is>
@@ -7299,7 +7591,7 @@
           <t>SLR-PLN-04, SLR-CLR-01, SLR-CLR-08, SLR-EXE-06</t>
         </is>
       </c>
-      <c r="F28" s="22" t="inlineStr">
+      <c r="F28" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7323,7 +7615,7 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>SN-PAX-02</t>
         </is>
@@ -7348,7 +7640,7 @@
           <t>SLR-MEA-03</t>
         </is>
       </c>
-      <c r="F29" s="22" t="inlineStr">
+      <c r="F29" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7372,7 +7664,7 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>SN-PAX-03</t>
         </is>
@@ -7397,7 +7689,7 @@
           <t>SLR-CLR-09, SLR-INF-06</t>
         </is>
       </c>
-      <c r="F30" s="22" t="inlineStr">
+      <c r="F30" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7421,7 +7713,7 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>SN-MIL-01</t>
         </is>
@@ -7446,7 +7738,7 @@
           <t>SLR-PLN-08, SLR-FLW-07, SLR-CLR-14</t>
         </is>
       </c>
-      <c r="F31" s="22" t="inlineStr">
+      <c r="F31" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -7585,7 +7877,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-01</t>
         </is>
@@ -7659,7 +7951,7 @@
       <c r="P2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-02</t>
         </is>
@@ -7733,7 +8025,7 @@
       <c r="P3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-04</t>
         </is>
@@ -7811,7 +8103,7 @@
       <c r="P4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-05</t>
         </is>
@@ -7885,7 +8177,7 @@
       <c r="P5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-06</t>
         </is>
@@ -7959,7 +8251,7 @@
       <c r="P6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-07</t>
         </is>
@@ -8033,7 +8325,7 @@
       <c r="P7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-08</t>
         </is>
@@ -8075,7 +8367,7 @@
         </is>
       </c>
       <c r="J8" s="13" t="inlineStr"/>
-      <c r="K8" s="22" t="inlineStr">
+      <c r="K8" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8103,7 +8395,7 @@
       <c r="P8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>SLR-PLN-09</t>
         </is>
@@ -8145,7 +8437,7 @@
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr"/>
-      <c r="K9" s="22" t="inlineStr">
+      <c r="K9" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8173,7 +8465,7 @@
       <c r="P9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>SLR-FLW-04</t>
         </is>
@@ -8215,7 +8507,7 @@
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr"/>
-      <c r="K10" s="22" t="inlineStr">
+      <c r="K10" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8243,7 +8535,7 @@
       <c r="P10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>SLR-FLW-05</t>
         </is>
@@ -8289,7 +8581,7 @@
           <t>assigned delay per flight, compared across airlines (minutes)</t>
         </is>
       </c>
-      <c r="K11" s="22" t="inlineStr">
+      <c r="K11" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8317,7 +8609,7 @@
       <c r="P11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>SLR-FLW-06</t>
         </is>
@@ -8363,7 +8655,7 @@
           <t>actual departure time minus EDCT (minutes)</t>
         </is>
       </c>
-      <c r="K12" s="22" t="inlineStr">
+      <c r="K12" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8391,7 +8683,7 @@
       <c r="P12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>SLR-FLW-07</t>
         </is>
@@ -8433,7 +8725,7 @@
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr"/>
-      <c r="K13" s="22" t="inlineStr">
+      <c r="K13" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8457,7 +8749,7 @@
       <c r="P13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-01</t>
         </is>
@@ -8535,7 +8827,7 @@
       <c r="P14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-02</t>
         </is>
@@ -8609,7 +8901,7 @@
       <c r="P15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-03</t>
         </is>
@@ -8651,7 +8943,7 @@
         </is>
       </c>
       <c r="J16" s="13" t="inlineStr"/>
-      <c r="K16" s="22" t="inlineStr">
+      <c r="K16" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8675,7 +8967,7 @@
       <c r="P16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-04</t>
         </is>
@@ -8745,7 +9037,7 @@
       <c r="P17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-05</t>
         </is>
@@ -8787,7 +9079,7 @@
         </is>
       </c>
       <c r="J18" s="13" t="inlineStr"/>
-      <c r="K18" s="22" t="inlineStr">
+      <c r="K18" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -8815,7 +9107,7 @@
       <c r="P18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-08</t>
         </is>
@@ -8889,7 +9181,7 @@
       <c r="P19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-09</t>
         </is>
@@ -8963,7 +9255,7 @@
       <c r="P20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-10</t>
         </is>
@@ -9037,7 +9329,7 @@
       <c r="P21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-13</t>
         </is>
@@ -9115,7 +9407,7 @@
       <c r="P22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-14</t>
         </is>
@@ -9157,7 +9449,7 @@
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr"/>
-      <c r="K23" s="22" t="inlineStr">
+      <c r="K23" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -9185,7 +9477,7 @@
       <c r="P23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>SLR-CLR-15</t>
         </is>
@@ -9263,7 +9555,7 @@
       <c r="P24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>SLR-INF-01</t>
         </is>
@@ -9337,7 +9629,7 @@
       <c r="P25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>SLR-INF-02</t>
         </is>
@@ -9411,7 +9703,7 @@
       <c r="P26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>SLR-INF-05</t>
         </is>
@@ -9453,7 +9745,7 @@
         </is>
       </c>
       <c r="J27" s="13" t="inlineStr"/>
-      <c r="K27" s="22" t="inlineStr">
+      <c r="K27" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -9481,7 +9773,7 @@
       <c r="P27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>SLR-INF-06</t>
         </is>
@@ -9523,7 +9815,7 @@
         </is>
       </c>
       <c r="J28" s="13" t="inlineStr"/>
-      <c r="K28" s="22" t="inlineStr">
+      <c r="K28" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -9551,7 +9843,7 @@
       <c r="P28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>SLR-INF-07</t>
         </is>
@@ -9629,7 +9921,7 @@
       <c r="P29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>SLR-EXE-01</t>
         </is>
@@ -9671,7 +9963,7 @@
         </is>
       </c>
       <c r="J30" s="13" t="inlineStr"/>
-      <c r="K30" s="22" t="inlineStr">
+      <c r="K30" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -9695,7 +9987,7 @@
       <c r="P30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>SLR-EXE-02</t>
         </is>
@@ -9769,7 +10061,7 @@
       <c r="P31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>SLR-EXE-03</t>
         </is>
@@ -9843,7 +10135,7 @@
       <c r="P32" s="13" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>SLR-EXE-04</t>
         </is>
@@ -9885,7 +10177,7 @@
         </is>
       </c>
       <c r="J33" s="13" t="inlineStr"/>
-      <c r="K33" s="22" t="inlineStr">
+      <c r="K33" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -9913,7 +10205,7 @@
       <c r="P33" s="13" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>SLR-EXE-06</t>
         </is>
@@ -9983,7 +10275,7 @@
       <c r="P34" s="13" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>SLR-APT-01</t>
         </is>
@@ -10025,7 +10317,7 @@
         </is>
       </c>
       <c r="J35" s="13" t="inlineStr"/>
-      <c r="K35" s="22" t="inlineStr">
+      <c r="K35" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -10049,7 +10341,7 @@
       <c r="P35" s="13" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="21" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>SLR-APT-02</t>
         </is>
@@ -10095,7 +10387,7 @@
           <t>runway operations per hour against the declared rate (operations per hour)</t>
         </is>
       </c>
-      <c r="K36" s="22" t="inlineStr">
+      <c r="K36" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -10123,7 +10415,7 @@
       <c r="P36" s="13" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>SLR-APT-03</t>
         </is>
@@ -10165,7 +10457,7 @@
         </is>
       </c>
       <c r="J37" s="13" t="inlineStr"/>
-      <c r="K37" s="22" t="inlineStr">
+      <c r="K37" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -10189,7 +10481,7 @@
       <c r="P37" s="13" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>SLR-APT-04</t>
         </is>
@@ -10267,7 +10559,7 @@
       <c r="P38" s="13" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>SLR-APT-05</t>
         </is>
@@ -10309,7 +10601,7 @@
         </is>
       </c>
       <c r="J39" s="13" t="inlineStr"/>
-      <c r="K39" s="22" t="inlineStr">
+      <c r="K39" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -10337,7 +10629,7 @@
       <c r="P39" s="13" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>SLR-MEA-01</t>
         </is>
@@ -10411,7 +10703,7 @@
       <c r="P40" s="13" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>SLR-MEA-02</t>
         </is>
@@ -10489,7 +10781,7 @@
       <c r="P41" s="13" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="23" t="inlineStr">
         <is>
           <t>SLR-MEA-03</t>
         </is>
@@ -10535,7 +10827,7 @@
           <t>gate arrival time minus scheduled arrival time (minutes)</t>
         </is>
       </c>
-      <c r="K42" s="22" t="inlineStr">
+      <c r="K42" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -10559,7 +10851,7 @@
       <c r="P42" s="13" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="23" t="inlineStr">
         <is>
           <t>SLR-MEA-04</t>
         </is>
@@ -10605,7 +10897,7 @@
           <t>assigned delay per flight (minutes)</t>
         </is>
       </c>
-      <c r="K43" s="22" t="inlineStr">
+      <c r="K43" s="24" t="inlineStr">
         <is>
           <t>outOfStudy</t>
         </is>
@@ -10750,7 +11042,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>HLR-CRW-01</t>
         </is>
@@ -10825,7 +11117,7 @@
       <c r="Q2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>HLR-CRW-02</t>
         </is>
@@ -10900,7 +11192,7 @@
       <c r="Q3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>HLR-CRW-03</t>
         </is>
@@ -10975,7 +11267,7 @@
       <c r="Q4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>HLR-CRW-04</t>
         </is>
@@ -11050,7 +11342,7 @@
       <c r="Q5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>HLR-CRW-05</t>
         </is>
@@ -11121,7 +11413,7 @@
       <c r="Q6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-01</t>
         </is>
@@ -11200,7 +11492,7 @@
       <c r="Q7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-02</t>
         </is>
@@ -11275,7 +11567,7 @@
       <c r="Q8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-03</t>
         </is>
@@ -11350,7 +11642,7 @@
       <c r="Q9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-04</t>
         </is>
@@ -11425,7 +11717,7 @@
       <c r="Q10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-05</t>
         </is>
@@ -11500,7 +11792,7 @@
       <c r="Q11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-06</t>
         </is>
@@ -11575,7 +11867,7 @@
       <c r="Q12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>HLR-OPS-07</t>
         </is>
@@ -11654,7 +11946,7 @@
       <c r="Q13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-01</t>
         </is>
@@ -11733,7 +12025,7 @@
       <c r="Q14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-02</t>
         </is>
@@ -11808,7 +12100,7 @@
       <c r="Q15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-03</t>
         </is>
@@ -11883,7 +12175,7 @@
       <c r="Q16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-04</t>
         </is>
@@ -11966,7 +12258,7 @@
       <c r="Q17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-05</t>
         </is>
@@ -12049,7 +12341,7 @@
       <c r="Q18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-06</t>
         </is>
@@ -12132,7 +12424,7 @@
       <c r="Q19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-07</t>
         </is>
@@ -12207,7 +12499,7 @@
       <c r="Q20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-08</t>
         </is>
@@ -12282,7 +12574,7 @@
       <c r="Q21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>HLR-ATC-09</t>
         </is>
@@ -12357,7 +12649,7 @@
       <c r="Q22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>HLR-ACF-01</t>
         </is>
@@ -12432,7 +12724,7 @@
       <c r="Q23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="23" t="inlineStr">
         <is>
           <t>HLR-ACF-02</t>
         </is>
@@ -12507,7 +12799,7 @@
       <c r="Q24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>HLR-ACF-03</t>
         </is>
@@ -12578,7 +12870,7 @@
       <c r="Q25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>HLR-ACF-04</t>
         </is>
@@ -12649,7 +12941,7 @@
       <c r="Q26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>HLR-ACF-05</t>
         </is>
@@ -12720,7 +13012,7 @@
       <c r="Q27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>HLR-ACF-06</t>
         </is>
@@ -12795,7 +13087,7 @@
       <c r="Q28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>HLR-APT-01</t>
         </is>
@@ -12874,7 +13166,7 @@
       <c r="Q29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>HLR-APT-02</t>
         </is>
@@ -12963,107 +13255,107 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Requirements review workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
-        <is>
-          <t>Generated 2026-10-22 21:42 from commit d0c723d by tools/export_requirements_xlsx.py.</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Generated 2026-10-27 17:40 from commit 574431f by tools/export_requirements_xlsx.py.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Source of truth: the .sysml files in projects/nas-sos-capstone/cameo_models/ (D-006). This workbook is a derived copy: mark it up, then apply the changes to the .sysml files and regenerate.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>Counts: 30 stakeholder requirements, 42 system requirements, 29 sub-system HLRs. The Coverage sheet counts each by scope and lists any trace gap.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr"/>
+      <c r="A5" s="27" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Objectives sheet: reads the other way, from each objective row of knowledge/models/stakeholder-objective-ontology.md to the stakeholder requirements that name it (attribute objectiveRefs), and on to the in-study system requirements and HLRs below them. Bold objective: carried into the study. Grey: carried only by a background or out-of-study requirement. '(no requirement)': no stakeholder requirement names it. Requirements that name no objective row are listed at the end.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr"/>
+      <c r="A7" s="27" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>How the Decomposition sheet reads</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Left to right: stakeholder requirement (SN) -&gt; the system requirements (SLR) that answer it -&gt; the HLRs that come from each SLR. Merged cells span the rows beneath them.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>The trace is many-to-many, so an SLR that answers two stakeholder requirements appears under both, marked '(also answers ...)'. An HLR with two parents is marked '(also comes from ...)'.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>[IMPROVED] and orange fill: architectureState = improved, something today's NAS does not do (D-018). [GOAL] and italics: obligation = goal, written with 'should' (D-020).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>[OUT OF STUDY], grey fill and grey text: studyScope = outOfStudy (D-031). Every stakeholder requirement of the first draft is kept, with the system requirements that answer it; the study's cut is made at the HLR tier, so these stop at the system level with '(no HLR: not carried into the study)'. [BACKGROUND] and lilac fill: a boundary actor's requirement the study holds fixed and uses as input (the operating rules, the CO2 factor). '(no HLR: gap)' in red would be an in-study system requirement with nothing under it.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr"/>
+      <c r="A13" s="27" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Review status (from knowledge/models/requirements-and-traceability.md)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>In-study stakeholder and system requirements: hand-reviewed by the owner three times (D-020, D-021, D-031). Out-of-study ones: restored on 2026-10-20 from the 10-10 and 10-11 prints with the text they had when struck.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>Sub-system HLRs: Claude's draft of 2026-10-11 (D-022), hand-reviewed by the owner on 2026-10-20 (D-031). Edits applied from a question on that print say so in their rationale and await the owner's confirmation; HLR-ACF-06 is new.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>Every requirement has status = draft. Nothing is baselined.</t>
         </is>

</xml_diff>